<commit_message>
Expand moveset coverage with GameBanana mods missing from UMC tracker
The compatibility tracker is opt-in, so it undercounts. Resolved host fighters
for GameBanana movesets by two additional methods: parsing slotting statements
in mod descriptions ("slotted ... beside Marth by default"), and following
companion-skin references to read their per-fighter category.

Adds Pikachu (Raichu), Lucario (Vegeta), Wolf (Zeraora), Little Mac (Naruto),
and Robin (Mona), plus second options for Dark Pit, Marth, Mewtwo, Ike and
Mega Man - including Gengar and Sasuke.

Coverage: 39 of 86 fighters (was 34), 14 with two options (was 12).

Adds per-suggestion confidence columns. Still excluded: non-slotted movesets
that overwrite a fighter globally (including Shadow, the game's most-liked
moveset), and reworks that alter the vanilla character instead of replacing it.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0137pZw7sF3W46xt4hxmpwDy
</commit_message>
<xml_diff>
--- a/smash_ultimate_moveset_mods.xlsx
+++ b/smash_ultimate_moveset_mods.xlsx
@@ -12,7 +12,7 @@
     <sheet name="Summary" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Moveset Mods'!$A$1:$K$87</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Moveset Mods'!$A$1:$L$87</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -166,10 +166,10 @@
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
@@ -537,23 +537,24 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K87"/>
+  <dimension ref="A1:L87"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
     <col width="22" customWidth="1" min="2" max="2"/>
-    <col width="46" customWidth="1" min="3" max="3"/>
+    <col width="44" customWidth="1" min="3" max="3"/>
     <col width="22" customWidth="1" min="4" max="4"/>
-    <col width="46" customWidth="1" min="5" max="5"/>
+    <col width="44" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
     <col width="12" customWidth="1" min="7" max="7"/>
     <col width="14" customWidth="1" min="8" max="8"/>
     <col width="14" customWidth="1" min="9" max="9"/>
-    <col width="26" customWidth="1" min="10" max="10"/>
-    <col width="34" customWidth="1" min="11" max="11"/>
+    <col width="30" customWidth="1" min="10" max="10"/>
+    <col width="30" customWidth="1" min="11" max="11"/>
+    <col width="30" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
-    <row r="1" ht="30" customHeight="1">
+    <row r="1" ht="32" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>original_char</t>
@@ -606,7 +607,12 @@
       </c>
       <c r="K1" s="1" t="inlineStr">
         <is>
-          <t>notes</t>
+          <t>sugg1_confidence</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>sugg2_confidence</t>
         </is>
       </c>
     </row>
@@ -649,7 +655,12 @@
           <t>single option available</t>
         </is>
       </c>
-      <c r="K2" s="6" t="inlineStr"/>
+      <c r="K2" s="6" t="inlineStr">
+        <is>
+          <t>verified (slots+hooks checked)</t>
+        </is>
+      </c>
+      <c r="L2" s="6" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="7" t="inlineStr">
@@ -704,7 +715,12 @@
       </c>
       <c r="K3" s="10" t="inlineStr">
         <is>
-          <t>sugg2 link = Discord server</t>
+          <t>verified (slots+hooks checked)</t>
+        </is>
+      </c>
+      <c r="L3" s="10" t="inlineStr">
+        <is>
+          <t>verified (slots+hooks checked)</t>
         </is>
       </c>
     </row>
@@ -736,6 +752,7 @@
         </is>
       </c>
       <c r="K4" s="14" t="inlineStr"/>
+      <c r="L4" s="14" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -776,7 +793,12 @@
           <t>single option available</t>
         </is>
       </c>
-      <c r="K5" s="6" t="inlineStr"/>
+      <c r="K5" s="6" t="inlineStr">
+        <is>
+          <t>verified (slots+hooks checked)</t>
+        </is>
+      </c>
+      <c r="L5" s="6" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="11" t="inlineStr">
@@ -806,6 +828,7 @@
         </is>
       </c>
       <c r="K6" s="14" t="inlineStr"/>
+      <c r="L6" s="14" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="11" t="inlineStr">
@@ -835,6 +858,7 @@
         </is>
       </c>
       <c r="K7" s="14" t="inlineStr"/>
+      <c r="L7" s="14" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="11" t="inlineStr">
@@ -864,6 +888,7 @@
         </is>
       </c>
       <c r="K8" s="14" t="inlineStr"/>
+      <c r="L8" s="14" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="11" t="inlineStr">
@@ -893,35 +918,53 @@
         </is>
       </c>
       <c r="K9" s="14" t="inlineStr"/>
+      <c r="L9" s="14" t="inlineStr"/>
     </row>
     <row r="10">
-      <c r="A10" s="11" t="inlineStr">
+      <c r="A10" s="2" t="inlineStr">
         <is>
           <t>Pikachu</t>
         </is>
       </c>
-      <c r="B10" s="12" t="inlineStr">
-        <is>
-          <t>NONE AVAILABLE</t>
-        </is>
-      </c>
-      <c r="C10" s="13" t="inlineStr"/>
-      <c r="D10" s="12" t="inlineStr">
-        <is>
-          <t>NONE AVAILABLE</t>
-        </is>
-      </c>
-      <c r="E10" s="13" t="inlineStr"/>
-      <c r="F10" s="13" t="inlineStr"/>
-      <c r="G10" s="13" t="inlineStr"/>
-      <c r="H10" s="13" t="inlineStr"/>
-      <c r="I10" s="13" t="inlineStr"/>
-      <c r="J10" s="14" t="inlineStr">
-        <is>
-          <t>no custom moveset exists</t>
-        </is>
-      </c>
-      <c r="K10" s="14" t="inlineStr"/>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>Raichu</t>
+        </is>
+      </c>
+      <c r="C10" s="4" t="inlineStr">
+        <is>
+          <t>https://gamebanana.com/mods/474333</t>
+        </is>
+      </c>
+      <c r="D10" s="5" t="inlineStr">
+        <is>
+          <t>NONE AVAILABLE</t>
+        </is>
+      </c>
+      <c r="E10" s="3" t="inlineStr"/>
+      <c r="F10" s="3" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="G10" s="3" t="inlineStr"/>
+      <c r="H10" s="3" t="inlineStr">
+        <is>
+          <t>Released</t>
+        </is>
+      </c>
+      <c r="I10" s="3" t="inlineStr"/>
+      <c r="J10" s="6" t="inlineStr">
+        <is>
+          <t>single option available</t>
+        </is>
+      </c>
+      <c r="K10" s="6" t="inlineStr">
+        <is>
+          <t>slotted ecosystem; slot range not published</t>
+        </is>
+      </c>
+      <c r="L10" s="6" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="11" t="inlineStr">
@@ -951,6 +994,7 @@
         </is>
       </c>
       <c r="K11" s="14" t="inlineStr"/>
+      <c r="L11" s="14" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="7" t="inlineStr">
@@ -1003,7 +1047,16 @@
           <t>verified conflict-free</t>
         </is>
       </c>
-      <c r="K12" s="10" t="inlineStr"/>
+      <c r="K12" s="10" t="inlineStr">
+        <is>
+          <t>verified (slots+hooks checked)</t>
+        </is>
+      </c>
+      <c r="L12" s="10" t="inlineStr">
+        <is>
+          <t>verified (slots+hooks checked)</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="7" t="inlineStr">
@@ -1056,7 +1109,16 @@
           <t>verified conflict-free</t>
         </is>
       </c>
-      <c r="K13" s="10" t="inlineStr"/>
+      <c r="K13" s="10" t="inlineStr">
+        <is>
+          <t>verified (slots+hooks checked)</t>
+        </is>
+      </c>
+      <c r="L13" s="10" t="inlineStr">
+        <is>
+          <t>verified (slots+hooks checked)</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="7" t="inlineStr">
@@ -1111,7 +1173,12 @@
       </c>
       <c r="K14" s="10" t="inlineStr">
         <is>
-          <t>joke mod</t>
+          <t>verified (slots+hooks checked)</t>
+        </is>
+      </c>
+      <c r="L14" s="10" t="inlineStr">
+        <is>
+          <t>verified (slots+hooks checked)</t>
         </is>
       </c>
     </row>
@@ -1156,9 +1223,10 @@
       </c>
       <c r="K15" s="6" t="inlineStr">
         <is>
-          <t>sugg1 link = UMC entry (no public mirror)</t>
-        </is>
-      </c>
+          <t>verified (slots+hooks checked)</t>
+        </is>
+      </c>
+      <c r="L15" s="6" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="11" t="inlineStr">
@@ -1188,6 +1256,7 @@
         </is>
       </c>
       <c r="K16" s="14" t="inlineStr"/>
+      <c r="L16" s="14" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -1228,7 +1297,12 @@
           <t>single option available</t>
         </is>
       </c>
-      <c r="K17" s="6" t="inlineStr"/>
+      <c r="K17" s="6" t="inlineStr">
+        <is>
+          <t>verified (slots+hooks checked)</t>
+        </is>
+      </c>
+      <c r="L17" s="6" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="11" t="inlineStr">
@@ -1258,6 +1332,7 @@
         </is>
       </c>
       <c r="K18" s="14" t="inlineStr"/>
+      <c r="L18" s="14" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="11" t="inlineStr">
@@ -1287,6 +1362,7 @@
         </is>
       </c>
       <c r="K19" s="14" t="inlineStr"/>
+      <c r="L19" s="14" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -1327,7 +1403,12 @@
           <t>single option available</t>
         </is>
       </c>
-      <c r="K20" s="6" t="inlineStr"/>
+      <c r="K20" s="6" t="inlineStr">
+        <is>
+          <t>verified (slots+hooks checked)</t>
+        </is>
+      </c>
+      <c r="L20" s="6" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" s="7" t="inlineStr">
@@ -1380,7 +1461,16 @@
           <t>verified conflict-free</t>
         </is>
       </c>
-      <c r="K21" s="10" t="inlineStr"/>
+      <c r="K21" s="10" t="inlineStr">
+        <is>
+          <t>verified (slots+hooks checked)</t>
+        </is>
+      </c>
+      <c r="L21" s="10" t="inlineStr">
+        <is>
+          <t>verified (slots+hooks checked)</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -1421,7 +1511,12 @@
           <t>single option available</t>
         </is>
       </c>
-      <c r="K22" s="6" t="inlineStr"/>
+      <c r="K22" s="6" t="inlineStr">
+        <is>
+          <t>verified (slots+hooks checked)</t>
+        </is>
+      </c>
+      <c r="L22" s="6" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -1462,7 +1557,12 @@
           <t>single option available</t>
         </is>
       </c>
-      <c r="K23" s="6" t="inlineStr"/>
+      <c r="K23" s="6" t="inlineStr">
+        <is>
+          <t>verified (slots+hooks checked)</t>
+        </is>
+      </c>
+      <c r="L23" s="6" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" s="7" t="inlineStr">
@@ -1517,7 +1617,12 @@
       </c>
       <c r="K24" s="10" t="inlineStr">
         <is>
-          <t>sugg2 link = UMC entry (no public mirror)</t>
+          <t>verified (slots+hooks checked)</t>
+        </is>
+      </c>
+      <c r="L24" s="10" t="inlineStr">
+        <is>
+          <t>verified (slots+hooks checked)</t>
         </is>
       </c>
     </row>
@@ -1549,6 +1654,7 @@
         </is>
       </c>
       <c r="K25" s="14" t="inlineStr"/>
+      <c r="L25" s="14" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" s="11" t="inlineStr">
@@ -1578,6 +1684,7 @@
         </is>
       </c>
       <c r="K26" s="14" t="inlineStr"/>
+      <c r="L26" s="14" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" s="7" t="inlineStr">
@@ -1630,7 +1737,16 @@
           <t>verified conflict-free</t>
         </is>
       </c>
-      <c r="K27" s="10" t="inlineStr"/>
+      <c r="K27" s="10" t="inlineStr">
+        <is>
+          <t>verified (slots+hooks checked)</t>
+        </is>
+      </c>
+      <c r="L27" s="10" t="inlineStr">
+        <is>
+          <t>verified (slots+hooks checked)</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="7" t="inlineStr">
@@ -1683,7 +1799,16 @@
           <t>verified conflict-free</t>
         </is>
       </c>
-      <c r="K28" s="10" t="inlineStr"/>
+      <c r="K28" s="10" t="inlineStr">
+        <is>
+          <t>verified (slots+hooks checked)</t>
+        </is>
+      </c>
+      <c r="L28" s="10" t="inlineStr">
+        <is>
+          <t>verified (slots+hooks checked)</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="11" t="inlineStr">
@@ -1713,6 +1838,7 @@
         </is>
       </c>
       <c r="K29" s="14" t="inlineStr"/>
+      <c r="L29" s="14" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
@@ -1753,7 +1879,12 @@
           <t>single option available</t>
         </is>
       </c>
-      <c r="K30" s="6" t="inlineStr"/>
+      <c r="K30" s="6" t="inlineStr">
+        <is>
+          <t>verified (slots+hooks checked)</t>
+        </is>
+      </c>
+      <c r="L30" s="6" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" s="11" t="inlineStr">
@@ -1783,6 +1914,7 @@
         </is>
       </c>
       <c r="K31" s="14" t="inlineStr"/>
+      <c r="L31" s="14" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
@@ -1825,9 +1957,10 @@
       </c>
       <c r="K32" s="6" t="inlineStr">
         <is>
-          <t>sugg1 link = Discord server</t>
-        </is>
-      </c>
+          <t>verified (slots+hooks checked)</t>
+        </is>
+      </c>
+      <c r="L32" s="6" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" s="11" t="inlineStr">
@@ -1857,47 +1990,69 @@
         </is>
       </c>
       <c r="K33" s="14" t="inlineStr"/>
+      <c r="L33" s="14" t="inlineStr"/>
     </row>
     <row r="34">
-      <c r="A34" s="2" t="inlineStr">
+      <c r="A34" s="7" t="inlineStr">
         <is>
           <t>Dark Pit</t>
         </is>
       </c>
-      <c r="B34" s="3" t="inlineStr">
+      <c r="B34" s="8" t="inlineStr">
         <is>
           <t>Krystal</t>
         </is>
       </c>
-      <c r="C34" s="4" t="inlineStr">
+      <c r="C34" s="9" t="inlineStr">
         <is>
           <t>https://gamebanana.com/mods/514829</t>
         </is>
       </c>
-      <c r="D34" s="5" t="inlineStr">
-        <is>
-          <t>NONE AVAILABLE</t>
-        </is>
-      </c>
-      <c r="E34" s="3" t="inlineStr"/>
-      <c r="F34" s="3" t="inlineStr">
+      <c r="D34" s="8" t="inlineStr">
+        <is>
+          <t>Decidueye</t>
+        </is>
+      </c>
+      <c r="E34" s="9" t="inlineStr">
+        <is>
+          <t>https://gamebanana.com/mods/513821</t>
+        </is>
+      </c>
+      <c r="F34" s="8" t="inlineStr">
         <is>
           <t>64-71</t>
         </is>
       </c>
-      <c r="G34" s="3" t="inlineStr"/>
-      <c r="H34" s="3" t="inlineStr">
-        <is>
-          <t>Released</t>
-        </is>
-      </c>
-      <c r="I34" s="3" t="inlineStr"/>
-      <c r="J34" s="6" t="inlineStr">
-        <is>
-          <t>single option available</t>
-        </is>
-      </c>
-      <c r="K34" s="6" t="inlineStr"/>
+      <c r="G34" s="8" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="H34" s="8" t="inlineStr">
+        <is>
+          <t>Released</t>
+        </is>
+      </c>
+      <c r="I34" s="8" t="inlineStr">
+        <is>
+          <t>Released</t>
+        </is>
+      </c>
+      <c r="J34" s="10" t="inlineStr">
+        <is>
+          <t>compatible stack; confirm slots on install</t>
+        </is>
+      </c>
+      <c r="K34" s="10" t="inlineStr">
+        <is>
+          <t>verified (slots+hooks checked)</t>
+        </is>
+      </c>
+      <c r="L34" s="10" t="inlineStr">
+        <is>
+          <t>slotted ecosystem; slot range not published</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="11" t="inlineStr">
@@ -1927,6 +2082,7 @@
         </is>
       </c>
       <c r="K35" s="14" t="inlineStr"/>
+      <c r="L35" s="14" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" s="11" t="inlineStr">
@@ -1956,6 +2112,7 @@
         </is>
       </c>
       <c r="K36" s="14" t="inlineStr"/>
+      <c r="L36" s="14" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" s="11" t="inlineStr">
@@ -1985,6 +2142,7 @@
         </is>
       </c>
       <c r="K37" s="14" t="inlineStr"/>
+      <c r="L37" s="14" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" s="7" t="inlineStr">
@@ -2037,7 +2195,16 @@
           <t>verified conflict-free</t>
         </is>
       </c>
-      <c r="K38" s="10" t="inlineStr"/>
+      <c r="K38" s="10" t="inlineStr">
+        <is>
+          <t>verified (slots+hooks checked)</t>
+        </is>
+      </c>
+      <c r="L38" s="10" t="inlineStr">
+        <is>
+          <t>verified (slots+hooks checked)</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="11" t="inlineStr">
@@ -2067,6 +2234,7 @@
         </is>
       </c>
       <c r="K39" s="14" t="inlineStr"/>
+      <c r="L39" s="14" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" s="11" t="inlineStr">
@@ -2096,6 +2264,7 @@
         </is>
       </c>
       <c r="K40" s="14" t="inlineStr"/>
+      <c r="L40" s="14" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
@@ -2136,7 +2305,12 @@
           <t>single option available</t>
         </is>
       </c>
-      <c r="K41" s="6" t="inlineStr"/>
+      <c r="K41" s="6" t="inlineStr">
+        <is>
+          <t>verified (slots+hooks checked)</t>
+        </is>
+      </c>
+      <c r="L41" s="6" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" s="7" t="inlineStr">
@@ -2189,7 +2363,16 @@
           <t>verified conflict-free</t>
         </is>
       </c>
-      <c r="K42" s="10" t="inlineStr"/>
+      <c r="K42" s="10" t="inlineStr">
+        <is>
+          <t>verified (slots+hooks checked)</t>
+        </is>
+      </c>
+      <c r="L42" s="10" t="inlineStr">
+        <is>
+          <t>verified (slots+hooks checked)</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="11" t="inlineStr">
@@ -2219,6 +2402,7 @@
         </is>
       </c>
       <c r="K43" s="14" t="inlineStr"/>
+      <c r="L43" s="14" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
@@ -2259,36 +2443,58 @@
           <t>single option available</t>
         </is>
       </c>
-      <c r="K44" s="6" t="inlineStr"/>
+      <c r="K44" s="6" t="inlineStr">
+        <is>
+          <t>verified (slots+hooks checked)</t>
+        </is>
+      </c>
+      <c r="L44" s="6" t="inlineStr"/>
     </row>
     <row r="45">
-      <c r="A45" s="11" t="inlineStr">
+      <c r="A45" s="2" t="inlineStr">
         <is>
           <t>Lucario</t>
         </is>
       </c>
-      <c r="B45" s="12" t="inlineStr">
-        <is>
-          <t>NONE AVAILABLE</t>
-        </is>
-      </c>
-      <c r="C45" s="13" t="inlineStr"/>
-      <c r="D45" s="12" t="inlineStr">
-        <is>
-          <t>NONE AVAILABLE</t>
-        </is>
-      </c>
-      <c r="E45" s="13" t="inlineStr"/>
-      <c r="F45" s="13" t="inlineStr"/>
-      <c r="G45" s="13" t="inlineStr"/>
-      <c r="H45" s="13" t="inlineStr"/>
-      <c r="I45" s="13" t="inlineStr"/>
-      <c r="J45" s="14" t="inlineStr">
-        <is>
-          <t>no custom moveset exists</t>
-        </is>
-      </c>
-      <c r="K45" s="14" t="inlineStr"/>
+      <c r="B45" s="3" t="inlineStr">
+        <is>
+          <t>Vegeta</t>
+        </is>
+      </c>
+      <c r="C45" s="4" t="inlineStr">
+        <is>
+          <t>https://gamebanana.com/mods/469216</t>
+        </is>
+      </c>
+      <c r="D45" s="5" t="inlineStr">
+        <is>
+          <t>NONE AVAILABLE</t>
+        </is>
+      </c>
+      <c r="E45" s="3" t="inlineStr"/>
+      <c r="F45" s="3" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="G45" s="3" t="inlineStr"/>
+      <c r="H45" s="3" t="inlineStr">
+        <is>
+          <t>Released</t>
+        </is>
+      </c>
+      <c r="I45" s="3" t="inlineStr"/>
+      <c r="J45" s="6" t="inlineStr">
+        <is>
+          <t>single option available</t>
+        </is>
+      </c>
+      <c r="K45" s="6" t="inlineStr">
+        <is>
+          <t>slotted ecosystem; slot range not published</t>
+        </is>
+      </c>
+      <c r="L45" s="6" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" s="11" t="inlineStr">
@@ -2318,6 +2524,7 @@
         </is>
       </c>
       <c r="K46" s="14" t="inlineStr"/>
+      <c r="L46" s="14" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" s="11" t="inlineStr">
@@ -2347,35 +2554,53 @@
         </is>
       </c>
       <c r="K47" s="14" t="inlineStr"/>
+      <c r="L47" s="14" t="inlineStr"/>
     </row>
     <row r="48">
-      <c r="A48" s="11" t="inlineStr">
+      <c r="A48" s="2" t="inlineStr">
         <is>
           <t>Wolf</t>
         </is>
       </c>
-      <c r="B48" s="12" t="inlineStr">
-        <is>
-          <t>NONE AVAILABLE</t>
-        </is>
-      </c>
-      <c r="C48" s="13" t="inlineStr"/>
-      <c r="D48" s="12" t="inlineStr">
-        <is>
-          <t>NONE AVAILABLE</t>
-        </is>
-      </c>
-      <c r="E48" s="13" t="inlineStr"/>
-      <c r="F48" s="13" t="inlineStr"/>
-      <c r="G48" s="13" t="inlineStr"/>
-      <c r="H48" s="13" t="inlineStr"/>
-      <c r="I48" s="13" t="inlineStr"/>
-      <c r="J48" s="14" t="inlineStr">
-        <is>
-          <t>no custom moveset exists</t>
-        </is>
-      </c>
-      <c r="K48" s="14" t="inlineStr"/>
+      <c r="B48" s="3" t="inlineStr">
+        <is>
+          <t>Zeraora</t>
+        </is>
+      </c>
+      <c r="C48" s="4" t="inlineStr">
+        <is>
+          <t>https://gamebanana.com/mods/524527</t>
+        </is>
+      </c>
+      <c r="D48" s="5" t="inlineStr">
+        <is>
+          <t>NONE AVAILABLE</t>
+        </is>
+      </c>
+      <c r="E48" s="3" t="inlineStr"/>
+      <c r="F48" s="3" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="G48" s="3" t="inlineStr"/>
+      <c r="H48" s="3" t="inlineStr">
+        <is>
+          <t>Released</t>
+        </is>
+      </c>
+      <c r="I48" s="3" t="inlineStr"/>
+      <c r="J48" s="6" t="inlineStr">
+        <is>
+          <t>single option available</t>
+        </is>
+      </c>
+      <c r="K48" s="6" t="inlineStr">
+        <is>
+          <t>slotted ecosystem; slot range not published</t>
+        </is>
+      </c>
+      <c r="L48" s="6" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
@@ -2416,48 +2641,74 @@
           <t>single option available</t>
         </is>
       </c>
-      <c r="K49" s="6" t="inlineStr"/>
+      <c r="K49" s="6" t="inlineStr">
+        <is>
+          <t>verified (slots+hooks checked)</t>
+        </is>
+      </c>
+      <c r="L49" s="6" t="inlineStr"/>
     </row>
     <row r="50">
-      <c r="A50" s="2" t="inlineStr">
+      <c r="A50" s="7" t="inlineStr">
         <is>
           <t>Mega Man</t>
         </is>
       </c>
-      <c r="B50" s="3" t="inlineStr">
+      <c r="B50" s="8" t="inlineStr">
         <is>
           <t>X</t>
         </is>
       </c>
-      <c r="C50" s="4" t="inlineStr">
+      <c r="C50" s="9" t="inlineStr">
         <is>
           <t>https://gamebanana.com/mods/605585</t>
         </is>
       </c>
-      <c r="D50" s="5" t="inlineStr">
-        <is>
-          <t>NONE AVAILABLE</t>
-        </is>
-      </c>
-      <c r="E50" s="3" t="inlineStr"/>
-      <c r="F50" s="3" t="inlineStr">
+      <c r="D50" s="8" t="inlineStr">
+        <is>
+          <t>Colette</t>
+        </is>
+      </c>
+      <c r="E50" s="9" t="inlineStr">
+        <is>
+          <t>https://gamebanana.com/mods/561040</t>
+        </is>
+      </c>
+      <c r="F50" s="8" t="inlineStr">
         <is>
           <t>95-102</t>
         </is>
       </c>
-      <c r="G50" s="3" t="inlineStr"/>
-      <c r="H50" s="3" t="inlineStr">
-        <is>
-          <t>Released</t>
-        </is>
-      </c>
-      <c r="I50" s="3" t="inlineStr"/>
-      <c r="J50" s="6" t="inlineStr">
-        <is>
-          <t>single option available</t>
-        </is>
-      </c>
-      <c r="K50" s="6" t="inlineStr"/>
+      <c r="G50" s="8" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="H50" s="8" t="inlineStr">
+        <is>
+          <t>Released</t>
+        </is>
+      </c>
+      <c r="I50" s="8" t="inlineStr">
+        <is>
+          <t>Released</t>
+        </is>
+      </c>
+      <c r="J50" s="10" t="inlineStr">
+        <is>
+          <t>compatible stack; confirm slots on install</t>
+        </is>
+      </c>
+      <c r="K50" s="10" t="inlineStr">
+        <is>
+          <t>verified (slots+hooks checked)</t>
+        </is>
+      </c>
+      <c r="L50" s="10" t="inlineStr">
+        <is>
+          <t>slotted ecosystem; slot range not published</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="11" t="inlineStr">
@@ -2487,6 +2738,7 @@
         </is>
       </c>
       <c r="K51" s="14" t="inlineStr"/>
+      <c r="L51" s="14" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" s="11" t="inlineStr">
@@ -2516,35 +2768,53 @@
         </is>
       </c>
       <c r="K52" s="14" t="inlineStr"/>
+      <c r="L52" s="14" t="inlineStr"/>
     </row>
     <row r="53">
-      <c r="A53" s="11" t="inlineStr">
+      <c r="A53" s="2" t="inlineStr">
         <is>
           <t>Little Mac</t>
         </is>
       </c>
-      <c r="B53" s="12" t="inlineStr">
-        <is>
-          <t>NONE AVAILABLE</t>
-        </is>
-      </c>
-      <c r="C53" s="13" t="inlineStr"/>
-      <c r="D53" s="12" t="inlineStr">
-        <is>
-          <t>NONE AVAILABLE</t>
-        </is>
-      </c>
-      <c r="E53" s="13" t="inlineStr"/>
-      <c r="F53" s="13" t="inlineStr"/>
-      <c r="G53" s="13" t="inlineStr"/>
-      <c r="H53" s="13" t="inlineStr"/>
-      <c r="I53" s="13" t="inlineStr"/>
-      <c r="J53" s="14" t="inlineStr">
-        <is>
-          <t>no custom moveset exists</t>
-        </is>
-      </c>
-      <c r="K53" s="14" t="inlineStr"/>
+      <c r="B53" s="3" t="inlineStr">
+        <is>
+          <t>Naruto Uzumaki</t>
+        </is>
+      </c>
+      <c r="C53" s="4" t="inlineStr">
+        <is>
+          <t>https://gamebanana.com/mods/478432</t>
+        </is>
+      </c>
+      <c r="D53" s="5" t="inlineStr">
+        <is>
+          <t>NONE AVAILABLE</t>
+        </is>
+      </c>
+      <c r="E53" s="3" t="inlineStr"/>
+      <c r="F53" s="3" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="G53" s="3" t="inlineStr"/>
+      <c r="H53" s="3" t="inlineStr">
+        <is>
+          <t>Released</t>
+        </is>
+      </c>
+      <c r="I53" s="3" t="inlineStr"/>
+      <c r="J53" s="6" t="inlineStr">
+        <is>
+          <t>single option available</t>
+        </is>
+      </c>
+      <c r="K53" s="6" t="inlineStr">
+        <is>
+          <t>slotted ecosystem; slot range not published</t>
+        </is>
+      </c>
+      <c r="L53" s="6" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
@@ -2585,7 +2855,12 @@
           <t>single option available</t>
         </is>
       </c>
-      <c r="K54" s="6" t="inlineStr"/>
+      <c r="K54" s="6" t="inlineStr">
+        <is>
+          <t>verified (slots+hooks checked)</t>
+        </is>
+      </c>
+      <c r="L54" s="6" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" s="11" t="inlineStr">
@@ -2615,6 +2890,7 @@
         </is>
       </c>
       <c r="K55" s="14" t="inlineStr"/>
+      <c r="L55" s="14" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" s="11" t="inlineStr">
@@ -2644,6 +2920,7 @@
         </is>
       </c>
       <c r="K56" s="14" t="inlineStr"/>
+      <c r="L56" s="14" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" s="11" t="inlineStr">
@@ -2673,6 +2950,7 @@
         </is>
       </c>
       <c r="K57" s="14" t="inlineStr"/>
+      <c r="L57" s="14" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" s="7" t="inlineStr">
@@ -2725,7 +3003,16 @@
           <t>verified conflict-free</t>
         </is>
       </c>
-      <c r="K58" s="10" t="inlineStr"/>
+      <c r="K58" s="10" t="inlineStr">
+        <is>
+          <t>verified (slots+hooks checked)</t>
+        </is>
+      </c>
+      <c r="L58" s="10" t="inlineStr">
+        <is>
+          <t>verified (slots+hooks checked)</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
@@ -2766,36 +3053,58 @@
           <t>single option available</t>
         </is>
       </c>
-      <c r="K59" s="6" t="inlineStr"/>
+      <c r="K59" s="6" t="inlineStr">
+        <is>
+          <t>verified (slots+hooks checked)</t>
+        </is>
+      </c>
+      <c r="L59" s="6" t="inlineStr"/>
     </row>
     <row r="60">
-      <c r="A60" s="11" t="inlineStr">
+      <c r="A60" s="2" t="inlineStr">
         <is>
           <t>Robin</t>
         </is>
       </c>
-      <c r="B60" s="12" t="inlineStr">
-        <is>
-          <t>NONE AVAILABLE</t>
-        </is>
-      </c>
-      <c r="C60" s="13" t="inlineStr"/>
-      <c r="D60" s="12" t="inlineStr">
-        <is>
-          <t>NONE AVAILABLE</t>
-        </is>
-      </c>
-      <c r="E60" s="13" t="inlineStr"/>
-      <c r="F60" s="13" t="inlineStr"/>
-      <c r="G60" s="13" t="inlineStr"/>
-      <c r="H60" s="13" t="inlineStr"/>
-      <c r="I60" s="13" t="inlineStr"/>
-      <c r="J60" s="14" t="inlineStr">
-        <is>
-          <t>no custom moveset exists</t>
-        </is>
-      </c>
-      <c r="K60" s="14" t="inlineStr"/>
+      <c r="B60" s="3" t="inlineStr">
+        <is>
+          <t>Mona</t>
+        </is>
+      </c>
+      <c r="C60" s="4" t="inlineStr">
+        <is>
+          <t>https://gamebanana.com/mods/533215</t>
+        </is>
+      </c>
+      <c r="D60" s="5" t="inlineStr">
+        <is>
+          <t>NONE AVAILABLE</t>
+        </is>
+      </c>
+      <c r="E60" s="3" t="inlineStr"/>
+      <c r="F60" s="3" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="G60" s="3" t="inlineStr"/>
+      <c r="H60" s="3" t="inlineStr">
+        <is>
+          <t>Released</t>
+        </is>
+      </c>
+      <c r="I60" s="3" t="inlineStr"/>
+      <c r="J60" s="6" t="inlineStr">
+        <is>
+          <t>single option available</t>
+        </is>
+      </c>
+      <c r="K60" s="6" t="inlineStr">
+        <is>
+          <t>slotted ecosystem; slot range not published</t>
+        </is>
+      </c>
+      <c r="L60" s="6" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" s="11" t="inlineStr">
@@ -2825,6 +3134,7 @@
         </is>
       </c>
       <c r="K61" s="14" t="inlineStr"/>
+      <c r="L61" s="14" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" s="11" t="inlineStr">
@@ -2854,6 +3164,7 @@
         </is>
       </c>
       <c r="K62" s="14" t="inlineStr"/>
+      <c r="L62" s="14" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" s="11" t="inlineStr">
@@ -2883,6 +3194,7 @@
         </is>
       </c>
       <c r="K63" s="14" t="inlineStr"/>
+      <c r="L63" s="14" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" s="11" t="inlineStr">
@@ -2912,6 +3224,7 @@
         </is>
       </c>
       <c r="K64" s="14" t="inlineStr"/>
+      <c r="L64" s="14" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
@@ -2952,7 +3265,12 @@
           <t>single option available</t>
         </is>
       </c>
-      <c r="K65" s="6" t="inlineStr"/>
+      <c r="K65" s="6" t="inlineStr">
+        <is>
+          <t>verified (slots+hooks checked)</t>
+        </is>
+      </c>
+      <c r="L65" s="6" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" s="11" t="inlineStr">
@@ -2982,6 +3300,7 @@
         </is>
       </c>
       <c r="K66" s="14" t="inlineStr"/>
+      <c r="L66" s="14" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
@@ -3024,9 +3343,10 @@
       </c>
       <c r="K67" s="6" t="inlineStr">
         <is>
-          <t>sugg1 link = UMC entry (no public mirror)</t>
-        </is>
-      </c>
+          <t>verified (slots+hooks checked)</t>
+        </is>
+      </c>
+      <c r="L67" s="6" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" s="11" t="inlineStr">
@@ -3056,6 +3376,7 @@
         </is>
       </c>
       <c r="K68" s="14" t="inlineStr"/>
+      <c r="L68" s="14" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" s="11" t="inlineStr">
@@ -3085,6 +3406,7 @@
         </is>
       </c>
       <c r="K69" s="14" t="inlineStr"/>
+      <c r="L69" s="14" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" s="11" t="inlineStr">
@@ -3114,6 +3436,7 @@
         </is>
       </c>
       <c r="K70" s="14" t="inlineStr"/>
+      <c r="L70" s="14" t="inlineStr"/>
     </row>
     <row r="71">
       <c r="A71" s="11" t="inlineStr">
@@ -3143,6 +3466,7 @@
         </is>
       </c>
       <c r="K71" s="14" t="inlineStr"/>
+      <c r="L71" s="14" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
@@ -3183,7 +3507,12 @@
           <t>single option available</t>
         </is>
       </c>
-      <c r="K72" s="6" t="inlineStr"/>
+      <c r="K72" s="6" t="inlineStr">
+        <is>
+          <t>verified (slots+hooks checked)</t>
+        </is>
+      </c>
+      <c r="L72" s="6" t="inlineStr"/>
     </row>
     <row r="73">
       <c r="A73" s="11" t="inlineStr">
@@ -3213,6 +3542,7 @@
         </is>
       </c>
       <c r="K73" s="14" t="inlineStr"/>
+      <c r="L73" s="14" t="inlineStr"/>
     </row>
     <row r="74">
       <c r="A74" s="11" t="inlineStr">
@@ -3242,6 +3572,7 @@
         </is>
       </c>
       <c r="K74" s="14" t="inlineStr"/>
+      <c r="L74" s="14" t="inlineStr"/>
     </row>
     <row r="75">
       <c r="A75" s="11" t="inlineStr">
@@ -3271,6 +3602,7 @@
         </is>
       </c>
       <c r="K75" s="14" t="inlineStr"/>
+      <c r="L75" s="14" t="inlineStr"/>
     </row>
     <row r="76">
       <c r="A76" s="11" t="inlineStr">
@@ -3300,6 +3632,7 @@
         </is>
       </c>
       <c r="K76" s="14" t="inlineStr"/>
+      <c r="L76" s="14" t="inlineStr"/>
     </row>
     <row r="77">
       <c r="A77" s="11" t="inlineStr">
@@ -3329,6 +3662,7 @@
         </is>
       </c>
       <c r="K77" s="14" t="inlineStr"/>
+      <c r="L77" s="14" t="inlineStr"/>
     </row>
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
@@ -3369,7 +3703,12 @@
           <t>single option available</t>
         </is>
       </c>
-      <c r="K78" s="6" t="inlineStr"/>
+      <c r="K78" s="6" t="inlineStr">
+        <is>
+          <t>verified (slots+hooks checked)</t>
+        </is>
+      </c>
+      <c r="L78" s="6" t="inlineStr"/>
     </row>
     <row r="79">
       <c r="A79" s="2" t="inlineStr">
@@ -3410,7 +3749,12 @@
           <t>single option available</t>
         </is>
       </c>
-      <c r="K79" s="6" t="inlineStr"/>
+      <c r="K79" s="6" t="inlineStr">
+        <is>
+          <t>verified (slots+hooks checked)</t>
+        </is>
+      </c>
+      <c r="L79" s="6" t="inlineStr"/>
     </row>
     <row r="80">
       <c r="A80" s="7" t="inlineStr">
@@ -3463,7 +3807,16 @@
           <t>verified conflict-free</t>
         </is>
       </c>
-      <c r="K80" s="10" t="inlineStr"/>
+      <c r="K80" s="10" t="inlineStr">
+        <is>
+          <t>verified (slots+hooks checked)</t>
+        </is>
+      </c>
+      <c r="L80" s="10" t="inlineStr">
+        <is>
+          <t>verified (slots+hooks checked)</t>
+        </is>
+      </c>
     </row>
     <row r="81">
       <c r="A81" s="11" t="inlineStr">
@@ -3493,6 +3846,7 @@
         </is>
       </c>
       <c r="K81" s="14" t="inlineStr"/>
+      <c r="L81" s="14" t="inlineStr"/>
     </row>
     <row r="82">
       <c r="A82" s="11" t="inlineStr">
@@ -3522,6 +3876,7 @@
         </is>
       </c>
       <c r="K82" s="14" t="inlineStr"/>
+      <c r="L82" s="14" t="inlineStr"/>
     </row>
     <row r="83">
       <c r="A83" s="11" t="inlineStr">
@@ -3551,6 +3906,7 @@
         </is>
       </c>
       <c r="K83" s="14" t="inlineStr"/>
+      <c r="L83" s="14" t="inlineStr"/>
     </row>
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
@@ -3591,7 +3947,12 @@
           <t>single option available</t>
         </is>
       </c>
-      <c r="K84" s="6" t="inlineStr"/>
+      <c r="K84" s="6" t="inlineStr">
+        <is>
+          <t>verified (slots+hooks checked)</t>
+        </is>
+      </c>
+      <c r="L84" s="6" t="inlineStr"/>
     </row>
     <row r="85">
       <c r="A85" s="11" t="inlineStr">
@@ -3621,6 +3982,7 @@
         </is>
       </c>
       <c r="K85" s="14" t="inlineStr"/>
+      <c r="L85" s="14" t="inlineStr"/>
     </row>
     <row r="86">
       <c r="A86" s="11" t="inlineStr">
@@ -3650,6 +4012,7 @@
         </is>
       </c>
       <c r="K86" s="14" t="inlineStr"/>
+      <c r="L86" s="14" t="inlineStr"/>
     </row>
     <row r="87">
       <c r="A87" s="11" t="inlineStr">
@@ -3679,56 +4042,64 @@
         </is>
       </c>
       <c r="K87" s="14" t="inlineStr"/>
+      <c r="L87" s="14" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:K87"/>
+  <autoFilter ref="A1:L87"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C3" r:id="rId2"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E3" r:id="rId3"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C5" r:id="rId4"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C12" r:id="rId5"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E12" r:id="rId6"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C13" r:id="rId7"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E13" r:id="rId8"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C14" r:id="rId9"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E14" r:id="rId10"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C15" r:id="rId11"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C17" r:id="rId12"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C20" r:id="rId13"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C21" r:id="rId14"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E21" r:id="rId15"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C22" r:id="rId16"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C23" r:id="rId17"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C24" r:id="rId18"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E24" r:id="rId19"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C27" r:id="rId20"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E27" r:id="rId21"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C28" r:id="rId22"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E28" r:id="rId23"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C30" r:id="rId24"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C32" r:id="rId25"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C34" r:id="rId26"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C38" r:id="rId27"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E38" r:id="rId28"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C41" r:id="rId29"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C42" r:id="rId30"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E42" r:id="rId31"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C44" r:id="rId32"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C49" r:id="rId33"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C50" r:id="rId34"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C54" r:id="rId35"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C58" r:id="rId36"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E58" r:id="rId37"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C59" r:id="rId38"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C65" r:id="rId39"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C67" r:id="rId40"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C72" r:id="rId41"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C78" r:id="rId42"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C79" r:id="rId43"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C80" r:id="rId44"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E80" r:id="rId45"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C84" r:id="rId46"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C10" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C12" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E12" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C13" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E13" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C14" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E14" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C15" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C17" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C20" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C21" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E21" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C22" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C23" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C24" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E24" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C27" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E27" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C28" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E28" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C30" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C32" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C34" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E34" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C38" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E38" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C41" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C42" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E42" r:id="rId33"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C44" r:id="rId34"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C45" r:id="rId35"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C48" r:id="rId36"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C49" r:id="rId37"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C50" r:id="rId38"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E50" r:id="rId39"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C53" r:id="rId40"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C54" r:id="rId41"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C58" r:id="rId42"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E58" r:id="rId43"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C59" r:id="rId44"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C60" r:id="rId45"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C65" r:id="rId46"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C67" r:id="rId47"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C72" r:id="rId48"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C78" r:id="rId49"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C79" r:id="rId50"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C80" r:id="rId51"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E80" r:id="rId52"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C84" r:id="rId53"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -3740,12 +4111,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C31"/>
+  <dimension ref="A1:B38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="118" customWidth="1" min="1" max="1"/>
     <col width="58" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -3774,128 +4144,88 @@
           <t>Download</t>
         </is>
       </c>
-      <c r="C4" s="17" t="inlineStr">
-        <is>
-          <t>Used by</t>
-        </is>
-      </c>
     </row>
     <row r="5">
-      <c r="A5" s="18" t="inlineStr">
+      <c r="A5" s="16" t="inlineStr">
         <is>
           <t>The CSK Collection</t>
         </is>
       </c>
-      <c r="B5" s="19" t="inlineStr">
+      <c r="B5" s="18" t="inlineStr">
         <is>
           <t>https://gamebanana.com/mods/499008</t>
         </is>
       </c>
-      <c r="C5" s="18" t="inlineStr">
-        <is>
-          <t>89/91</t>
-        </is>
-      </c>
     </row>
     <row r="6">
-      <c r="A6" s="18" t="inlineStr">
+      <c r="A6" s="16" t="inlineStr">
         <is>
           <t>NRO Hook</t>
         </is>
       </c>
-      <c r="B6" s="19" t="inlineStr">
+      <c r="B6" s="18" t="inlineStr">
         <is>
           <t>https://github.com/ultimate-research/nro-hook-plugin/releases</t>
         </is>
       </c>
-      <c r="C6" s="18" t="inlineStr">
-        <is>
-          <t>89/91</t>
-        </is>
-      </c>
     </row>
     <row r="7">
-      <c r="A7" s="18" t="inlineStr">
+      <c r="A7" s="16" t="inlineStr">
         <is>
           <t>Smashline 2</t>
         </is>
       </c>
-      <c r="B7" s="19" t="inlineStr">
+      <c r="B7" s="18" t="inlineStr">
         <is>
           <t>https://github.com/HDR-Development/smashline</t>
         </is>
       </c>
-      <c r="C7" s="18" t="inlineStr">
-        <is>
-          <t>89/91</t>
-        </is>
-      </c>
     </row>
     <row r="8">
-      <c r="A8" s="18" t="inlineStr">
+      <c r="A8" s="16" t="inlineStr">
         <is>
           <t>ARCropolis</t>
         </is>
       </c>
-      <c r="B8" s="19" t="inlineStr">
+      <c r="B8" s="18" t="inlineStr">
         <is>
           <t>https://github.com/Raytwo/ARCropolis</t>
         </is>
       </c>
-      <c r="C8" s="18" t="inlineStr">
-        <is>
-          <t>88/91</t>
-        </is>
-      </c>
     </row>
     <row r="9">
-      <c r="A9" s="18" t="inlineStr">
+      <c r="A9" s="16" t="inlineStr">
         <is>
           <t>Skyline</t>
         </is>
       </c>
-      <c r="B9" s="19" t="inlineStr">
+      <c r="B9" s="18" t="inlineStr">
         <is>
           <t>https://github.com/skyline-dev/skyline</t>
         </is>
       </c>
-      <c r="C9" s="18" t="inlineStr">
-        <is>
-          <t>88/91</t>
-        </is>
-      </c>
     </row>
     <row r="10">
-      <c r="A10" s="18" t="inlineStr">
+      <c r="A10" s="16" t="inlineStr">
         <is>
           <t>paramconfig</t>
         </is>
       </c>
-      <c r="B10" s="19" t="inlineStr">
+      <c r="B10" s="18" t="inlineStr">
         <is>
           <t>https://github.com/CSharpM7/lib_paramconfig</t>
         </is>
       </c>
-      <c r="C10" s="18" t="inlineStr">
-        <is>
-          <t>88/91</t>
-        </is>
-      </c>
     </row>
     <row r="11">
-      <c r="A11" s="18" t="inlineStr">
+      <c r="A11" s="16" t="inlineStr">
         <is>
           <t>One Slot Effects</t>
         </is>
       </c>
-      <c r="B11" s="19" t="inlineStr">
+      <c r="B11" s="18" t="inlineStr">
         <is>
           <t>https://gamebanana.com/mods/549058</t>
-        </is>
-      </c>
-      <c r="C11" s="18" t="inlineStr">
-        <is>
-          <t>78/91</t>
         </is>
       </c>
     </row>
@@ -3903,119 +4233,162 @@
     <row r="13">
       <c r="A13" s="16" t="inlineStr">
         <is>
+          <t>CONFIDENCE LEVELS (see sugg1_confidence / sugg2_confidence)</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="16" t="inlineStr">
+        <is>
+          <t>'verified (slots+hooks checked)' - tracked in the Ultimate Moveset Compatibility database. Costume slot range and</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    hooked memory offsets are published, so conflicts were checked programmatically. Highest confidence.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="16" t="inlineStr">
+        <is>
+          <t>'slotted ecosystem; slot range not published' - GameBanana mod confirmed to use the CSK slotting method / Smashline 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    (same plugin stack), but its slot range is not published, so overlap could not be auto-verified. Confirm on install.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18"/>
+    <row r="19">
+      <c r="A19" s="19" t="inlineStr">
+        <is>
           <t>WHY THESE MODS ARE INTERCOMPATIBLE</t>
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="18" t="inlineStr">
-        <is>
-          <t>1. Every listed moveset is SLOTTED: it occupies a specific costume-slot range (columns sugg1_slots / sugg2_slots)</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="18" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    instead of replacing the fighter globally. Two movesets on one fighter coexist when their slot ranges differ.</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="18" t="inlineStr">
-        <is>
-          <t>2. All are built on the same Smashline 2 + ARCropolis stack above, so they share one plugin set instead of conflicting ones.</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="18" t="inlineStr">
-        <is>
-          <t>3. Each pair below was checked programmatically for (a) slot-range overlap, (b) shared hooked memory offsets,</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="18" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    and (c) both using a global 'opff' (once-per-frame) hook. Only conflict-free pairs were selected.</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="18" t="inlineStr">
-        <is>
-          <t>4. AVOID non-slotted / older movesets (typical pre-Smashline-2 GameBanana uploads): they overwrite the entire fighter and</t>
-        </is>
-      </c>
-    </row>
     <row r="20">
-      <c r="A20" s="18" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    break every other mod on that character. That constraint is why this list is limited to the slotted ecosystem.</t>
+      <c r="A20" s="16" t="inlineStr">
+        <is>
+          <t>1. Every listed moveset is SLOTTED: it occupies specific costume slots rather than replacing the fighter globally,</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="18" t="inlineStr">
-        <is>
-          <t>5. If you ever hit a slot overlap, ranges can be reassigned with a reslotter tool.</t>
+      <c r="A21" s="16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    so several can coexist. Two movesets on one fighter are fine as long as their slot ranges differ.</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="18" t="inlineStr">
-        <is>
-          <t>6. Movesets are not Wi-Fi safe - use them offline / in local play only.</t>
-        </is>
-      </c>
-    </row>
-    <row r="23"/>
+      <c r="A22" s="16" t="inlineStr">
+        <is>
+          <t>2. All share the Smashline 2 + ARCropolis + CSK stack above - one plugin set, not competing ones.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="16" t="inlineStr">
+        <is>
+          <t>3. Tier-A pairs were checked for slot-range overlap, shared hooked memory offsets, and concurrent global 'opff' hooks.</t>
+        </is>
+      </c>
+    </row>
     <row r="24">
       <c r="A24" s="16" t="inlineStr">
         <is>
-          <t>SCOPE / COVERAGE</t>
+          <t>4. EXCLUDED: non-slotted movesets, which overwrite the whole fighter and break every other mod on it. The most popular</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="18" t="inlineStr">
-        <is>
-          <t>Only 34 of 86 fighters have a released slotted custom moveset; 12 have two. Remaining fighters have none in existence.</t>
+      <c r="A25" s="16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    moveset in the game (Shadow the Hedgehog, 465 likes) is excluded for exactly this reason - it states no slotting.</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="18" t="inlineStr">
-        <is>
-          <t>Roster uses the 86 in-game fighter slots (Pokemon Trainer = 1 entry, Pyra / Mythra = 1 entry).</t>
+      <c r="A26" s="16" t="inlineStr">
+        <is>
+          <t>5. Also excluded: reworks of a vanilla fighter (Sonic Re-Imagined, Dread Samus, Swole Luigi). They change the original</t>
         </is>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="18" t="inlineStr">
-        <is>
-          <t>'NONE AVAILABLE' means no such mod exists - not that it was omitted.</t>
-        </is>
-      </c>
-    </row>
-    <row r="28"/>
+      <c r="A27" s="16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    character rather than replacing them, so they do not answer 'which mod character replaces X'.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="16" t="inlineStr">
+        <is>
+          <t>6. Slot ranges can be reassigned with a reslotter tool if you hit an overlap.</t>
+        </is>
+      </c>
+    </row>
     <row r="29">
       <c r="A29" s="16" t="inlineStr">
         <is>
-          <t>SOURCES</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="19" t="inlineStr">
-        <is>
-          <t>https://lilylavender.github.io/UltimateMovesetCompatibility/</t>
-        </is>
-      </c>
-    </row>
+          <t>7. Movesets are NOT Wi-Fi safe - offline / local play only.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30"/>
     <row r="31">
       <c r="A31" s="19" t="inlineStr">
+        <is>
+          <t>COVERAGE</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="16" t="inlineStr">
+        <is>
+          <t>39 of 86 fighters have at least one custom moveset; 14 have two. 47 have none in existence.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="16" t="inlineStr">
+        <is>
+          <t>'NONE AVAILABLE' means no such mod has been made - not that it was omitted.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="16" t="inlineStr">
+        <is>
+          <t>Roster = 86 in-game fighter slots (Pokemon Trainer = 1 entry, Pyra / Mythra = 1 entry).</t>
+        </is>
+      </c>
+    </row>
+    <row r="35"/>
+    <row r="36">
+      <c r="A36" s="19" t="inlineStr">
+        <is>
+          <t>SOURCES</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="18" t="inlineStr">
+        <is>
+          <t>https://lilylavender.github.io/UltimateMovesetCompatibility/</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="18" t="inlineStr">
         <is>
           <t>https://gamebanana.com/mods/cats/3325</t>
         </is>
@@ -4030,8 +4403,8 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B9" r:id="rId5"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B10" r:id="rId6"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B11" r:id="rId7"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A30" r:id="rId8"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A31" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A37" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A38" r:id="rId9"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -4076,7 +4449,7 @@
     <row r="3">
       <c r="A3" s="21" t="inlineStr">
         <is>
-          <t>Fighters with at least 1 custom moveset</t>
+          <t>Fighters with at least 1 moveset</t>
         </is>
       </c>
       <c r="B3" s="21">
@@ -4098,7 +4471,7 @@
     <row r="5">
       <c r="A5" s="21" t="inlineStr">
         <is>
-          <t>Fighters with NO custom moveset</t>
+          <t>Fighters with NO moveset</t>
         </is>
       </c>
       <c r="B5" s="21">

</xml_diff>